<commit_message>
reran calculate metrics after cell type fix
</commit_message>
<xml_diff>
--- a/Output Files GPT-OSS 20B/metrics_summary_gptoss.xlsx
+++ b/Output Files GPT-OSS 20B/metrics_summary_gptoss.xlsx
@@ -3995,7 +3995,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>3.46</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="180">
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>54</v>
+        <v>1</v>
       </c>
     </row>
     <row r="181">
@@ -4055,7 +4055,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>0.2769</v>
+        <v>0.0051</v>
       </c>
     </row>
     <row r="183">
@@ -4075,7 +4075,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>0.2769</v>
+        <v>0.1282</v>
       </c>
     </row>
     <row r="184">
@@ -4115,7 +4115,7 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>54</v>
+        <v>25</v>
       </c>
     </row>
     <row r="186">

</xml_diff>